<commit_message>
update with minor changes in historical flood data
</commit_message>
<xml_diff>
--- a/flood_data/Bhutan_Historical_Floods_1979_2025.xlsx
+++ b/flood_data/Bhutan_Historical_Floods_1979_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuq13/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuq13/bhutan_climate_modeling/flood_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{C26341DF-5CF2-D249-BE79-CE228D40593C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06E85B70-C3A1-F64F-8736-491B30C70898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1280" yWindow="820" windowWidth="28040" windowHeight="17080" xr2:uid="{F55684F5-72B6-D349-A1EC-EF84D62D24E3}"/>
+    <workbookView xWindow="1280" yWindow="820" windowWidth="33400" windowHeight="18800" xr2:uid="{F55684F5-72B6-D349-A1EC-EF84D62D24E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Bhutan_Historical_Floods" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="170">
   <si>
     <t>Date</t>
   </si>
@@ -64,9 +64,6 @@
     <t>Flash Flood</t>
   </si>
   <si>
-    <t>Flash flood</t>
-  </si>
-  <si>
     <t>Sarpang</t>
   </si>
   <si>
@@ -76,48 +73,24 @@
     <t>Flood</t>
   </si>
   <si>
-    <t>Monsoon flood</t>
-  </si>
-  <si>
     <t>Phuentsholing</t>
   </si>
   <si>
-    <t>Major flood</t>
-  </si>
-  <si>
-    <t>Urban flooding</t>
-  </si>
-  <si>
     <t>Flood swept through the market</t>
   </si>
   <si>
-    <t>Major monsoon flood: roads destroyed</t>
-  </si>
-  <si>
-    <t>Flash flood in town</t>
-  </si>
-  <si>
     <t>Floods swept away houses and crops</t>
   </si>
   <si>
     <t>Samdrup Jongkhar</t>
   </si>
   <si>
-    <t>Flash flood caused by heavy rain</t>
-  </si>
-  <si>
-    <t>Cyclone Aila: Major floods in southern Bhutan</t>
-  </si>
-  <si>
     <t>Thimphu</t>
   </si>
   <si>
     <t>Olarongchu, Babesa, Hongtsho</t>
   </si>
   <si>
-    <t>FLOOD</t>
-  </si>
-  <si>
     <t>1. Nar Bdr was washed away by Olarongchu on 26th May, 2009. The body is still not recovered 2. Tandin Wangmo was washed away by Hongtsho stream on [...]</t>
   </si>
   <si>
@@ -136,9 +109,6 @@
     <t>Taktichu, Papaling,</t>
   </si>
   <si>
-    <t>1. The labourer was washed away by landslide 2. Ms. Narim was washed away by flash flood during cattle migration to Paro (Body recovered and [...]</t>
-  </si>
-  <si>
     <t>Metakha</t>
   </si>
   <si>
@@ -262,9 +232,6 @@
     <t>Samtse, Chukha, Sarpang</t>
   </si>
   <si>
-    <t>Continuous heavy rain caused flash floods and landslides</t>
-  </si>
-  <si>
     <t>Continuous</t>
   </si>
   <si>
@@ -277,12 +244,6 @@
     <t>Lhuentse town</t>
   </si>
   <si>
-    <t>Flash flood due to monsoon rains</t>
-  </si>
-  <si>
-    <t>Flash flood and urban flooding</t>
-  </si>
-  <si>
     <t>Flooding caused traffic standstill</t>
   </si>
   <si>
@@ -298,18 +259,9 @@
     <t>Kholong Chu, Manas</t>
   </si>
   <si>
-    <t>Nakpola and Kukturgang caused flash flood</t>
-  </si>
-  <si>
-    <t>Flash flood following intense rain</t>
-  </si>
-  <si>
     <t>Khomachhu, Manas</t>
   </si>
   <si>
-    <t>Swollen stream caused flood</t>
-  </si>
-  <si>
     <t>Mangdichhu, Manas</t>
   </si>
   <si>
@@ -319,9 +271,6 @@
     <t>Phuntsharge, Sankosh</t>
   </si>
   <si>
-    <t>Heavy rain caused flash flood</t>
-  </si>
-  <si>
     <t>Gelephu</t>
   </si>
   <si>
@@ -334,9 +283,6 @@
     <t>Mao River, Aichhu</t>
   </si>
   <si>
-    <t>Heavy rain caused flood</t>
-  </si>
-  <si>
     <t>Cherichhu, Wangchu</t>
   </si>
   <si>
@@ -352,12 +298,6 @@
     <t>Dhaula River</t>
   </si>
   <si>
-    <t>Heavy rainfall caused urban flooding</t>
-  </si>
-  <si>
-    <t>Urban flooding due to intense rainfall</t>
-  </si>
-  <si>
     <t>Tsirang</t>
   </si>
   <si>
@@ -370,9 +310,6 @@
     <t>Mithimdrang stream, Manas</t>
   </si>
   <si>
-    <t>Small flash floods reported; heavy rain mainly in eastern Bhutan</t>
-  </si>
-  <si>
     <t>Daily accumulation</t>
   </si>
   <si>
@@ -403,9 +340,6 @@
     <t>Bjizam</t>
   </si>
   <si>
-    <t>Flash flood caused six families to lose homes and damaged bridge</t>
-  </si>
-  <si>
     <t>Chamdey Gangchu Stream, Manas</t>
   </si>
   <si>
@@ -424,9 +358,6 @@
     <t>Ruecheykha</t>
   </si>
   <si>
-    <t>Flash flood destroyed crops</t>
-  </si>
-  <si>
     <t>Puntsangchu</t>
   </si>
   <si>
@@ -436,9 +367,6 @@
     <t>Chendebji, Trongsa</t>
   </si>
   <si>
-    <t>Flash flood caused minor damage to bridge, houses, and logs</t>
-  </si>
-  <si>
     <t>Prior hours</t>
   </si>
   <si>
@@ -448,12 +376,6 @@
     <t>Chendebji</t>
   </si>
   <si>
-    <t>Flash flood destroyed bridge</t>
-  </si>
-  <si>
-    <t>Flash flood and landslide</t>
-  </si>
-  <si>
     <t>Trashiyangtse</t>
   </si>
   <si>
@@ -481,9 +403,6 @@
     <t>Trongsa town</t>
   </si>
   <si>
-    <t>Urban flooding after heavy rainfall</t>
-  </si>
-  <si>
     <t>Pemagatshel</t>
   </si>
   <si>
@@ -508,37 +427,109 @@
     <t>Phuentshogling (Toorsa, Kabreytar and nearby areas)</t>
   </si>
   <si>
-    <t>a flash flood around 5:30¬†AM flooded ten National Housing Development Corporation units and five private units and affected shops; another flash flood around 7:30¬†AM in Kabreytar washed away a car; landslides occurred in upper Kabreytar and behind a multi‚Äëlevel car park, washing away the Pasakha road</t>
-  </si>
-  <si>
     <t>Oong‚Äëgar (Ungar) Chiwog, Maedtsho Gewog, Lhuentse</t>
   </si>
   <si>
-    <t>It washed away 23 people including De‚Äësuup trainees and Druk Green Power Corporation workers; six bodies were recovered while the rest were missing; the flood also swept away camps, machines, vehicles, about 10 cattle and paddy fields</t>
-  </si>
-  <si>
     <t>Thangu Chiwog, Wangdue Phodrang</t>
   </si>
   <si>
-    <t>Continuous rainfall raised water levels in the Punatsangchhu, flooding Thangu village on 25¬†August¬†2023; five houses and about five acres of paddy field were submerged, damaging rice grains stored on ground floors; water also flooded a brick factory and staff quarters below Rinchengang.</t>
-  </si>
-  <si>
     <t>Dechencholing (Dangrina area), Thimphu</t>
   </si>
   <si>
-    <t>Heavy rainfall triggered a flood and landslide in Dechencholing; the flood split the stream into three channels, damaging the Dangrina bridge and roads, and uprooted trees; roads were impassable and officials were clearing debris</t>
-  </si>
-  <si>
     <t>Punakha‚ÄëGasa highway (Geyza Chhura Lum, Domey Lum and Tago Lum)</t>
   </si>
   <si>
-    <t>heavy rain triggered flash floods that washed away sections of the Punakha‚ÄëGasa highway at Geyza Chhura¬†Lum, Domey¬†Lum and Tago¬†Lum, leaving Gasa district cut off; authorities planned a temporary bypass and reported no casualties.</t>
-  </si>
-  <si>
     <t>Damkhi‚ÄëRinakha Chiwog, Toebisa Gewog, Punakha</t>
   </si>
   <si>
-    <t>A flash flood from the Phetsiri stream at Tendrel Lum washed away the only access road to Damkhi‚ÄëRinakha Chiwog; heavy rainfall caused the flood, cutting off the community of more than 40 households and disrupting transport of essential goods</t>
+    <t>Monsoon Flood</t>
+  </si>
+  <si>
+    <t>Major Flood</t>
+  </si>
+  <si>
+    <t>Urban Flooding</t>
+  </si>
+  <si>
+    <t>Major monsoon Flood: roads destroyed</t>
+  </si>
+  <si>
+    <t>Flash Flood in town</t>
+  </si>
+  <si>
+    <t>Flash Flood caused by heavy rain</t>
+  </si>
+  <si>
+    <t>Cyclone Aila: Major Floods in southern Bhutan</t>
+  </si>
+  <si>
+    <t>1. The labourer was washed away by landslide 2. Ms. Narim was washed away by flash Flood during cattle migration to Paro (Body recovered and [...]</t>
+  </si>
+  <si>
+    <t>Continuous heavy rain caused flash Floods and landslides</t>
+  </si>
+  <si>
+    <t>Flash Flood due to monsoon rains</t>
+  </si>
+  <si>
+    <t>Flash Flood and urban Flooding</t>
+  </si>
+  <si>
+    <t>Flash Flood following intense rain</t>
+  </si>
+  <si>
+    <t>Swollen stream caused Flood</t>
+  </si>
+  <si>
+    <t>Heavy rain caused flash Flood</t>
+  </si>
+  <si>
+    <t>Heavy rain caused Flood</t>
+  </si>
+  <si>
+    <t>Heavy rainfall caused urban Flooding</t>
+  </si>
+  <si>
+    <t>Urban Flooding due to intense rainfall</t>
+  </si>
+  <si>
+    <t>Small flash Floods reported; heavy rain mainly in eastern Bhutan</t>
+  </si>
+  <si>
+    <t>Flash Flood caused six families to lose homes and damaged bridge</t>
+  </si>
+  <si>
+    <t>Flash Flood destroyed crops</t>
+  </si>
+  <si>
+    <t>Flash Flood caused minor damage to bridge, houses, and logs</t>
+  </si>
+  <si>
+    <t>Flash Flood destroyed bridge</t>
+  </si>
+  <si>
+    <t>Flash Flood and landslide</t>
+  </si>
+  <si>
+    <t>Urban Flooding after heavy rainfall</t>
+  </si>
+  <si>
+    <t>a flash Flood around 5:30¬†AM Flooded ten National Housing Development Corporation units and five private units and affected shops; another flash Flood around 7:30¬†AM in Kabreytar washed away a car; landslides occurred in upper Kabreytar and behind a multi‚Äëlevel car park, washing away the Pasakha road</t>
+  </si>
+  <si>
+    <t>It washed away 23 people including De‚Äësuup trainees and Druk Green Power Corporation workers; six bodies were recovered while the rest were missing; the Flood also swept away camps, machines, vehicles, about 10 cattle and paddy fields</t>
+  </si>
+  <si>
+    <t>Continuous rainfall raised water levels in the Punatsangchhu, Flooding Thangu village on 25¬†August¬†2023; five houses and about five acres of paddy field were submerged, damaging rice grains stored on ground floors; water also Flooded a brick factory and staff quarters below Rinchengang.</t>
+  </si>
+  <si>
+    <t>Heavy rainfall triggered a Flood and landslide in Dechencholing; the Flood split the stream into three channels, damaging the Dangrina bridge and roads, and uprooted trees; roads were impassable and officials were clearing debris</t>
+  </si>
+  <si>
+    <t>heavy rain triggered flash Floods that washed away sections of the Punakha‚ÄëGasa highway at Geyza Chhura¬†Lum, Domey¬†Lum and Tago¬†Lum, leaving Gasa district cut off; authorities planned a temporary bypass and reported no casualties.</t>
+  </si>
+  <si>
+    <t>A flash Flood from the Phetsiri stream at Tendrel Lum washed away the only access road to Damkhi‚ÄëRinakha Chiwog; heavy rainfall caused the Flood, cutting off the community of more than 40 households and disrupting transport of essential goods</t>
   </si>
 </sst>
 </file>
@@ -1402,6 +1393,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E12EF590-DE3E-884F-8F1C-0835A05DDFF5}">
   <dimension ref="A1:K114"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="6" max="6" width="35.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -1458,7 +1452,7 @@
         <v>13</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1469,10 +1463,10 @@
         <v>33093</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D3">
         <v>26.8627</v>
@@ -1484,7 +1478,7 @@
         <v>13</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K3">
         <v>1</v>
@@ -1495,10 +1489,10 @@
         <v>34525</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D4">
         <v>27.5916</v>
@@ -1507,10 +1501,10 @@
         <v>89.877399999999994</v>
       </c>
       <c r="F4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G4" t="s">
-        <v>18</v>
+        <v>140</v>
       </c>
       <c r="K4">
         <v>1</v>
@@ -1521,10 +1515,10 @@
         <v>35291</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D5">
         <v>26.863499999999998</v>
@@ -1533,10 +1527,10 @@
         <v>89.388300000000001</v>
       </c>
       <c r="F5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G5" t="s">
-        <v>20</v>
+        <v>141</v>
       </c>
       <c r="K5">
         <v>1</v>
@@ -1547,10 +1541,10 @@
         <v>36723</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D6">
         <v>26.863499999999998</v>
@@ -1559,10 +1553,10 @@
         <v>89.388300000000001</v>
       </c>
       <c r="F6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G6" t="s">
-        <v>21</v>
+        <v>142</v>
       </c>
       <c r="K6">
         <v>1</v>
@@ -1573,10 +1567,10 @@
         <v>36750</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D7">
         <v>26.8627</v>
@@ -1588,7 +1582,7 @@
         <v>13</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="K7">
         <v>1</v>
@@ -1599,10 +1593,10 @@
         <v>38193</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D8">
         <v>26.8627</v>
@@ -1611,10 +1605,10 @@
         <v>90.271699999999996</v>
       </c>
       <c r="F8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G8" t="s">
-        <v>23</v>
+        <v>143</v>
       </c>
       <c r="K8">
         <v>1</v>
@@ -1625,10 +1619,10 @@
         <v>38194</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D9">
         <v>26.863499999999998</v>
@@ -1637,10 +1631,10 @@
         <v>89.388300000000001</v>
       </c>
       <c r="F9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G9" t="s">
-        <v>24</v>
+        <v>144</v>
       </c>
       <c r="K9">
         <v>1</v>
@@ -1651,10 +1645,10 @@
         <v>38917</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D10">
         <v>27.5916</v>
@@ -1666,7 +1660,7 @@
         <v>13</v>
       </c>
       <c r="G10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K10">
         <v>1</v>
@@ -1677,10 +1671,10 @@
         <v>39278</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D11">
         <v>26.8627</v>
@@ -1689,10 +1683,10 @@
         <v>90.271699999999996</v>
       </c>
       <c r="F11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G11" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="K11">
         <v>1</v>
@@ -1703,10 +1697,10 @@
         <v>39652</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D12">
         <v>26.805499999999999</v>
@@ -1718,7 +1712,7 @@
         <v>13</v>
       </c>
       <c r="G12" t="s">
-        <v>27</v>
+        <v>145</v>
       </c>
       <c r="K12">
         <v>1</v>
@@ -1729,10 +1723,10 @@
         <v>39958</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D13">
         <v>26.8627</v>
@@ -1741,10 +1735,10 @@
         <v>90.271699999999996</v>
       </c>
       <c r="F13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G13" t="s">
-        <v>28</v>
+        <v>146</v>
       </c>
       <c r="K13">
         <v>1</v>
@@ -1755,10 +1749,10 @@
         <v>39989</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D14">
         <v>27.466090000000001</v>
@@ -1767,13 +1761,13 @@
         <v>89.641909999999996</v>
       </c>
       <c r="F14" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G14" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I14" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="K14">
         <v>2</v>
@@ -1784,7 +1778,7 @@
         <v>39989</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D15">
         <v>27.5916</v>
@@ -1793,13 +1787,13 @@
         <v>89.877399999999994</v>
       </c>
       <c r="F15" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G15" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="I15" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="K15">
         <v>2</v>
@@ -1810,10 +1804,10 @@
         <v>39989</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="C16" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D16">
         <v>27.078430399999998</v>
@@ -1822,13 +1816,13 @@
         <v>89.474217699999997</v>
       </c>
       <c r="F16" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G16" t="s">
-        <v>38</v>
+        <v>147</v>
       </c>
       <c r="I16" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="K16">
         <v>2</v>
@@ -1839,10 +1833,10 @@
         <v>39989</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="D17">
         <v>27.641839000000001</v>
@@ -1851,13 +1845,13 @@
         <v>90.677304599999999</v>
       </c>
       <c r="F17" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G17" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="I17" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="K17">
         <v>2</v>
@@ -1877,13 +1871,13 @@
         <v>89.899500000000003</v>
       </c>
       <c r="F18" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G18" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="I18" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="K18">
         <v>2</v>
@@ -1894,7 +1888,7 @@
         <v>39989</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D19">
         <v>27.265166900000001</v>
@@ -1903,13 +1897,13 @@
         <v>89.170599800000005</v>
       </c>
       <c r="F19" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G19" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="I19" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="K19">
         <v>2</v>
@@ -1920,10 +1914,10 @@
         <v>39989</v>
       </c>
       <c r="B20" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C20" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D20">
         <v>28.051500000000001</v>
@@ -1932,13 +1926,13 @@
         <v>89.634299999999996</v>
       </c>
       <c r="F20" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G20" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="I20" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="K20">
         <v>2</v>
@@ -1949,7 +1943,7 @@
         <v>39989</v>
       </c>
       <c r="B21" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="D21">
         <v>27.530100000000001</v>
@@ -1958,10 +1952,10 @@
         <v>90.548950000000005</v>
       </c>
       <c r="F21" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G21" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="K21">
         <v>2</v>
@@ -1972,10 +1966,10 @@
         <v>40384</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C22" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="D22">
         <v>26.899699999999999</v>
@@ -1984,10 +1978,10 @@
         <v>89.101100000000002</v>
       </c>
       <c r="F22" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G22" t="s">
-        <v>18</v>
+        <v>140</v>
       </c>
       <c r="K22">
         <v>1</v>
@@ -1998,10 +1992,10 @@
         <v>40396</v>
       </c>
       <c r="B23" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C23" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="D23">
         <v>27.333200000000001</v>
@@ -2013,7 +2007,7 @@
         <v>13</v>
       </c>
       <c r="G23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K23">
         <v>1</v>
@@ -2024,10 +2018,10 @@
         <v>40732</v>
       </c>
       <c r="B24" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C24" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="D24">
         <v>26.863499999999998</v>
@@ -2036,10 +2030,10 @@
         <v>89.388300000000001</v>
       </c>
       <c r="F24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K24">
         <v>1</v>
@@ -2050,7 +2044,7 @@
         <v>40789</v>
       </c>
       <c r="B25" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D25">
         <v>27.466090000000001</v>
@@ -2059,10 +2053,10 @@
         <v>89.641909999999996</v>
       </c>
       <c r="F25" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="I25" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="K25">
         <v>2</v>
@@ -2073,10 +2067,10 @@
         <v>41109</v>
       </c>
       <c r="B26" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C26" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D26">
         <v>26.8627</v>
@@ -2088,7 +2082,7 @@
         <v>13</v>
       </c>
       <c r="G26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K26">
         <v>1</v>
@@ -2099,7 +2093,7 @@
         <v>41370</v>
       </c>
       <c r="B27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D27">
         <v>27.5916</v>
@@ -2108,13 +2102,13 @@
         <v>89.877399999999994</v>
       </c>
       <c r="F27" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G27" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="I27" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="K27">
         <v>2</v>
@@ -2125,10 +2119,10 @@
         <v>41502</v>
       </c>
       <c r="B28" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C28" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D28">
         <v>27.5916</v>
@@ -2140,7 +2134,7 @@
         <v>13</v>
       </c>
       <c r="G28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K28">
         <v>1</v>
@@ -2151,10 +2145,10 @@
         <v>41504</v>
       </c>
       <c r="B29" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C29" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D29">
         <v>26.805499999999999</v>
@@ -2163,10 +2157,10 @@
         <v>91.503600000000006</v>
       </c>
       <c r="F29" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G29" t="s">
-        <v>21</v>
+        <v>142</v>
       </c>
       <c r="K29">
         <v>1</v>
@@ -2177,7 +2171,7 @@
         <v>41623</v>
       </c>
       <c r="B30" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D30">
         <v>27.5916</v>
@@ -2186,10 +2180,10 @@
         <v>89.877399999999994</v>
       </c>
       <c r="F30" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="I30" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="K30">
         <v>2</v>
@@ -2200,7 +2194,7 @@
         <v>41688</v>
       </c>
       <c r="B31" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D31">
         <v>27.5916</v>
@@ -2209,10 +2203,10 @@
         <v>89.877399999999994</v>
       </c>
       <c r="F31" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="I31" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="K31">
         <v>2</v>
@@ -2223,7 +2217,7 @@
         <v>41717</v>
       </c>
       <c r="B32" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D32">
         <v>27.097003399999998</v>
@@ -2232,13 +2226,13 @@
         <v>89.873898699999998</v>
       </c>
       <c r="F32" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G32" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="I32" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="K32">
         <v>2</v>
@@ -2249,10 +2243,10 @@
         <v>41717</v>
       </c>
       <c r="B33" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="C33" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="D33">
         <v>26.803568200000001</v>
@@ -2261,13 +2255,13 @@
         <v>91.503920699999995</v>
       </c>
       <c r="F33" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G33" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="I33" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="K33">
         <v>2</v>
@@ -2278,10 +2272,10 @@
         <v>41826</v>
       </c>
       <c r="B34" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C34" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="D34">
         <v>26.863499999999998</v>
@@ -2290,10 +2284,10 @@
         <v>89.388300000000001</v>
       </c>
       <c r="F34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G34" t="s">
-        <v>18</v>
+        <v>140</v>
       </c>
       <c r="K34">
         <v>1</v>
@@ -2304,10 +2298,10 @@
         <v>42197</v>
       </c>
       <c r="B35" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="C35" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="D35">
         <v>27.267600000000002</v>
@@ -2316,13 +2310,13 @@
         <v>91.193100000000001</v>
       </c>
       <c r="F35" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G35" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="I35" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="K35">
         <v>2</v>
@@ -2333,10 +2327,10 @@
         <v>42210</v>
       </c>
       <c r="B36" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="D36">
         <v>28.051500000000001</v>
@@ -2348,7 +2342,7 @@
         <v>13</v>
       </c>
       <c r="G36" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K36">
         <v>1</v>
@@ -2359,10 +2353,10 @@
         <v>42225</v>
       </c>
       <c r="B37" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C37" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D37">
         <v>26.8627</v>
@@ -2371,10 +2365,10 @@
         <v>90.271699999999996</v>
       </c>
       <c r="F37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K37">
         <v>1</v>
@@ -2385,10 +2379,10 @@
         <v>42241</v>
       </c>
       <c r="B38" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C38" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="D38">
         <v>26.899699999999999</v>
@@ -2397,10 +2391,10 @@
         <v>89.101100000000002</v>
       </c>
       <c r="F38" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G38" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K38">
         <v>1</v>
@@ -2411,7 +2405,7 @@
         <v>42300</v>
       </c>
       <c r="B39" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D39">
         <v>27.5916</v>
@@ -2420,13 +2414,13 @@
         <v>89.877399999999994</v>
       </c>
       <c r="F39" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G39" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="I39" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="K39">
         <v>2</v>
@@ -2437,10 +2431,10 @@
         <v>42566</v>
       </c>
       <c r="B40" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C40" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="D40">
         <v>27.029183199999999</v>
@@ -2452,10 +2446,10 @@
         <v>13</v>
       </c>
       <c r="G40" t="s">
-        <v>80</v>
+        <v>148</v>
       </c>
       <c r="H40" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="K40">
         <v>3</v>
@@ -2466,10 +2460,10 @@
         <v>42566</v>
       </c>
       <c r="B41" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C41" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="D41">
         <v>26.867899999999999</v>
@@ -2481,10 +2475,10 @@
         <v>13</v>
       </c>
       <c r="G41" t="s">
-        <v>80</v>
+        <v>148</v>
       </c>
       <c r="H41" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="K41">
         <v>3</v>
@@ -2495,10 +2489,10 @@
         <v>42566</v>
       </c>
       <c r="B42" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="C42" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="D42">
         <v>27.078430399999998</v>
@@ -2510,10 +2504,10 @@
         <v>13</v>
       </c>
       <c r="G42" t="s">
-        <v>80</v>
+        <v>148</v>
       </c>
       <c r="H42" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="K42">
         <v>3</v>
@@ -2524,10 +2518,10 @@
         <v>42570</v>
       </c>
       <c r="B43" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C43" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="D43">
         <v>27.6678</v>
@@ -2539,7 +2533,7 @@
         <v>13</v>
       </c>
       <c r="G43" t="s">
-        <v>85</v>
+        <v>149</v>
       </c>
       <c r="K43">
         <v>1</v>
@@ -2550,10 +2544,10 @@
         <v>42571</v>
       </c>
       <c r="B44" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C44" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D44">
         <v>26.805499999999999</v>
@@ -2565,7 +2559,7 @@
         <v>13</v>
       </c>
       <c r="G44" t="s">
-        <v>86</v>
+        <v>150</v>
       </c>
       <c r="K44">
         <v>1</v>
@@ -2576,10 +2570,10 @@
         <v>42585</v>
       </c>
       <c r="B45" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C45" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="D45">
         <v>26.863499999999998</v>
@@ -2588,10 +2582,10 @@
         <v>89.388300000000001</v>
       </c>
       <c r="F45" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G45" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="K45">
         <v>1</v>
@@ -2602,10 +2596,10 @@
         <v>42850</v>
       </c>
       <c r="B46" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C46" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D46">
         <v>28.051500000000001</v>
@@ -2617,7 +2611,7 @@
         <v>13</v>
       </c>
       <c r="J46" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="K46">
         <v>4</v>
@@ -2628,10 +2622,10 @@
         <v>42860</v>
       </c>
       <c r="B47" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C47" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D47">
         <v>27.333200000000001</v>
@@ -2643,7 +2637,7 @@
         <v>13</v>
       </c>
       <c r="J47" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="K47">
         <v>4</v>
@@ -2654,10 +2648,10 @@
         <v>42912</v>
       </c>
       <c r="B48" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="C48" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="D48">
         <v>27.611599999999999</v>
@@ -2666,10 +2660,10 @@
         <v>91.498000000000005</v>
       </c>
       <c r="F48" t="s">
-        <v>92</v>
+        <v>13</v>
       </c>
       <c r="J48" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="K48">
         <v>4</v>
@@ -2680,10 +2674,10 @@
         <v>42928</v>
       </c>
       <c r="B49" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C49" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D49">
         <v>26.8627</v>
@@ -2695,7 +2689,7 @@
         <v>13</v>
       </c>
       <c r="G49" t="s">
-        <v>93</v>
+        <v>151</v>
       </c>
       <c r="K49">
         <v>1</v>
@@ -2706,10 +2700,10 @@
         <v>42933</v>
       </c>
       <c r="B50" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C50" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="D50">
         <v>27.6678</v>
@@ -2718,10 +2712,13 @@
         <v>91.183000000000007</v>
       </c>
       <c r="F50" t="s">
-        <v>95</v>
+        <v>16</v>
+      </c>
+      <c r="G50" t="s">
+        <v>152</v>
       </c>
       <c r="J50" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="K50">
         <v>4</v>
@@ -2732,10 +2729,10 @@
         <v>42934</v>
       </c>
       <c r="B51" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C51" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="D51">
         <v>27.530100000000001</v>
@@ -2747,7 +2744,7 @@
         <v>13</v>
       </c>
       <c r="J51" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="K51">
         <v>4</v>
@@ -2758,10 +2755,10 @@
         <v>42938</v>
       </c>
       <c r="B52" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="C52" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="D52">
         <v>27.452604600000001</v>
@@ -2770,10 +2767,13 @@
         <v>90.067492799999997</v>
       </c>
       <c r="F52" t="s">
-        <v>99</v>
+        <v>13</v>
+      </c>
+      <c r="G52" t="s">
+        <v>153</v>
       </c>
       <c r="J52" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="K52">
         <v>4</v>
@@ -2784,10 +2784,10 @@
         <v>42944</v>
       </c>
       <c r="B53" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C53" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D53">
         <v>27.6678</v>
@@ -2796,10 +2796,13 @@
         <v>91.183000000000007</v>
       </c>
       <c r="F53" t="s">
-        <v>99</v>
+        <v>13</v>
+      </c>
+      <c r="G53" t="s">
+        <v>153</v>
       </c>
       <c r="J53" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="K53">
         <v>4</v>
@@ -2810,10 +2813,10 @@
         <v>42955</v>
       </c>
       <c r="B54" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="C54" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="D54">
         <v>26.870556000000001</v>
@@ -2825,7 +2828,7 @@
         <v>13</v>
       </c>
       <c r="J54" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="K54">
         <v>4</v>
@@ -2836,10 +2839,10 @@
         <v>42956</v>
       </c>
       <c r="B55" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C55" t="s">
-        <v>102</v>
+        <v>85</v>
       </c>
       <c r="D55">
         <v>27.5916</v>
@@ -2848,10 +2851,10 @@
         <v>89.877399999999994</v>
       </c>
       <c r="F55" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J55" t="s">
-        <v>102</v>
+        <v>85</v>
       </c>
       <c r="K55">
         <v>4</v>
@@ -2862,10 +2865,10 @@
         <v>42957</v>
       </c>
       <c r="B56" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="C56" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="D56">
         <v>26.870556000000001</v>
@@ -2874,10 +2877,13 @@
         <v>90.485557999999997</v>
       </c>
       <c r="F56" t="s">
-        <v>104</v>
+        <v>16</v>
+      </c>
+      <c r="G56" t="s">
+        <v>154</v>
       </c>
       <c r="J56" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="K56">
         <v>4</v>
@@ -2888,10 +2894,10 @@
         <v>42960</v>
       </c>
       <c r="B57" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C57" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="D57">
         <v>27.466090000000001</v>
@@ -2900,10 +2906,13 @@
         <v>89.641909999999996</v>
       </c>
       <c r="F57" t="s">
-        <v>106</v>
+        <v>13</v>
+      </c>
+      <c r="G57" t="s">
+        <v>88</v>
       </c>
       <c r="J57" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="K57">
         <v>4</v>
@@ -2914,10 +2923,10 @@
         <v>42962</v>
       </c>
       <c r="B58" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C58" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D58">
         <v>27.5916</v>
@@ -2926,10 +2935,10 @@
         <v>89.877399999999994</v>
       </c>
       <c r="F58" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G58" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="K58">
         <v>1</v>
@@ -2940,10 +2949,10 @@
         <v>42977</v>
       </c>
       <c r="B59" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="C59" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="D59">
         <v>26.870556000000001</v>
@@ -2955,7 +2964,7 @@
         <v>13</v>
       </c>
       <c r="J59" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="K59">
         <v>4</v>
@@ -2966,10 +2975,10 @@
         <v>42982</v>
       </c>
       <c r="B60" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C60" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="D60">
         <v>26.8627</v>
@@ -2978,10 +2987,13 @@
         <v>90.271699999999996</v>
       </c>
       <c r="F60" t="s">
-        <v>104</v>
+        <v>16</v>
+      </c>
+      <c r="G60" t="s">
+        <v>154</v>
       </c>
       <c r="J60" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="K60">
         <v>4</v>
@@ -2992,10 +3004,10 @@
         <v>43020</v>
       </c>
       <c r="B61" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="C61" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D61">
         <v>27.267600000000002</v>
@@ -3004,10 +3016,10 @@
         <v>91.193100000000001</v>
       </c>
       <c r="F61" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J61" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="K61">
         <v>4</v>
@@ -3018,10 +3030,10 @@
         <v>43264</v>
       </c>
       <c r="B62" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C62" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D62">
         <v>27.6678</v>
@@ -3030,10 +3042,10 @@
         <v>91.183000000000007</v>
       </c>
       <c r="F62" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J62" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="K62">
         <v>4</v>
@@ -3044,10 +3056,10 @@
         <v>43291</v>
       </c>
       <c r="B63" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C63" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D63">
         <v>26.863499999999998</v>
@@ -3056,10 +3068,10 @@
         <v>89.388300000000001</v>
       </c>
       <c r="F63" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G63" t="s">
-        <v>110</v>
+        <v>155</v>
       </c>
       <c r="K63">
         <v>1</v>
@@ -3070,10 +3082,10 @@
         <v>43301</v>
       </c>
       <c r="B64" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C64" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D64">
         <v>26.805499999999999</v>
@@ -3082,10 +3094,10 @@
         <v>91.503600000000006</v>
       </c>
       <c r="F64" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G64" t="s">
-        <v>111</v>
+        <v>156</v>
       </c>
       <c r="K64">
         <v>1</v>
@@ -3096,10 +3108,10 @@
         <v>43301</v>
       </c>
       <c r="B65" t="s">
-        <v>112</v>
+        <v>92</v>
       </c>
       <c r="C65" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="D65">
         <v>27.0246</v>
@@ -3108,10 +3120,10 @@
         <v>90.124600000000001</v>
       </c>
       <c r="F65" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G65" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="K65">
         <v>1</v>
@@ -3122,10 +3134,10 @@
         <v>43303</v>
       </c>
       <c r="B66" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C66" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="D66">
         <v>27.333200000000001</v>
@@ -3137,7 +3149,7 @@
         <v>13</v>
       </c>
       <c r="J66" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="K66">
         <v>4</v>
@@ -3148,10 +3160,10 @@
         <v>43313</v>
       </c>
       <c r="B67" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C67" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="D67">
         <v>27.333200000000001</v>
@@ -3163,7 +3175,7 @@
         <v>13</v>
       </c>
       <c r="G67" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K67">
         <v>1</v>
@@ -3174,10 +3186,10 @@
         <v>43319</v>
       </c>
       <c r="B68" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C68" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="D68">
         <v>26.899699999999999</v>
@@ -3189,7 +3201,7 @@
         <v>13</v>
       </c>
       <c r="G68" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K68">
         <v>1</v>
@@ -3200,10 +3212,10 @@
         <v>43584</v>
       </c>
       <c r="B69" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C69" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="D69">
         <v>27.667870000000001</v>
@@ -3215,10 +3227,10 @@
         <v>13</v>
       </c>
       <c r="G69" t="s">
-        <v>116</v>
+        <v>157</v>
       </c>
       <c r="H69" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="K69">
         <v>3</v>
@@ -3229,10 +3241,10 @@
         <v>43584</v>
       </c>
       <c r="B70" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C70" t="s">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="D70">
         <v>27.6678</v>
@@ -3244,7 +3256,7 @@
         <v>13</v>
       </c>
       <c r="J70" t="s">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="K70">
         <v>4</v>
@@ -3255,10 +3267,10 @@
         <v>43642</v>
       </c>
       <c r="B71" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="C71" t="s">
-        <v>119</v>
+        <v>98</v>
       </c>
       <c r="D71">
         <v>27.267600000000002</v>
@@ -3270,7 +3282,7 @@
         <v>13</v>
       </c>
       <c r="G71" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K71">
         <v>1</v>
@@ -3281,10 +3293,10 @@
         <v>43651</v>
       </c>
       <c r="B72" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C72" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D72">
         <v>26.8627</v>
@@ -3296,7 +3308,7 @@
         <v>13</v>
       </c>
       <c r="G72" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K72">
         <v>1</v>
@@ -3307,10 +3319,10 @@
         <v>43671</v>
       </c>
       <c r="B73" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C73" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D73">
         <v>27.6678</v>
@@ -3322,7 +3334,7 @@
         <v>13</v>
       </c>
       <c r="J73" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="K73">
         <v>4</v>
@@ -3333,10 +3345,10 @@
         <v>43672</v>
       </c>
       <c r="B74" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="C74" t="s">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="D74">
         <v>27.078430399999998</v>
@@ -3348,7 +3360,7 @@
         <v>13</v>
       </c>
       <c r="J74" t="s">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="K74">
         <v>4</v>
@@ -3359,10 +3371,10 @@
         <v>43683</v>
       </c>
       <c r="B75" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C75" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="D75">
         <v>27.5916</v>
@@ -3371,10 +3383,10 @@
         <v>89.877399999999994</v>
       </c>
       <c r="F75" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J75" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="K75">
         <v>4</v>
@@ -3385,10 +3397,10 @@
         <v>43684</v>
       </c>
       <c r="B76" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="C76" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="D76">
         <v>27.452604600000001</v>
@@ -3400,10 +3412,10 @@
         <v>13</v>
       </c>
       <c r="G76" t="s">
-        <v>123</v>
+        <v>102</v>
       </c>
       <c r="H76" t="s">
-        <v>124</v>
+        <v>103</v>
       </c>
       <c r="K76">
         <v>3</v>
@@ -3414,10 +3426,10 @@
         <v>44032</v>
       </c>
       <c r="B77" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="C77" t="s">
-        <v>125</v>
+        <v>104</v>
       </c>
       <c r="D77">
         <v>26.870556000000001</v>
@@ -3426,10 +3438,10 @@
         <v>90.485557999999997</v>
       </c>
       <c r="F77" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J77" t="s">
-        <v>125</v>
+        <v>104</v>
       </c>
       <c r="K77">
         <v>4</v>
@@ -3440,10 +3452,10 @@
         <v>44105</v>
       </c>
       <c r="B78" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C78" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="D78">
         <v>27.500226999999999</v>
@@ -3455,10 +3467,10 @@
         <v>13</v>
       </c>
       <c r="G78" t="s">
-        <v>127</v>
+        <v>158</v>
       </c>
       <c r="H78" t="s">
-        <v>124</v>
+        <v>103</v>
       </c>
       <c r="K78">
         <v>3</v>
@@ -3469,10 +3481,10 @@
         <v>44105</v>
       </c>
       <c r="B79" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C79" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="D79">
         <v>27.530100000000001</v>
@@ -3484,7 +3496,7 @@
         <v>13</v>
       </c>
       <c r="J79" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="K79">
         <v>4</v>
@@ -3495,10 +3507,10 @@
         <v>44105</v>
       </c>
       <c r="B80" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
       <c r="C80" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="D80">
         <v>27.215800000000002</v>
@@ -3510,7 +3522,7 @@
         <v>13</v>
       </c>
       <c r="G80" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K80">
         <v>1</v>
@@ -3521,10 +3533,10 @@
         <v>44108</v>
       </c>
       <c r="B81" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="C81" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="D81">
         <v>27.486149999999999</v>
@@ -3536,10 +3548,10 @@
         <v>13</v>
       </c>
       <c r="G81" t="s">
-        <v>131</v>
+        <v>109</v>
       </c>
       <c r="H81" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
       <c r="K81">
         <v>3</v>
@@ -3553,7 +3565,7 @@
         <v>11</v>
       </c>
       <c r="C82" t="s">
-        <v>133</v>
+        <v>111</v>
       </c>
       <c r="D82">
         <v>27.430599999999998</v>
@@ -3565,7 +3577,7 @@
         <v>13</v>
       </c>
       <c r="G82" t="s">
-        <v>134</v>
+        <v>159</v>
       </c>
       <c r="K82">
         <v>1</v>
@@ -3576,10 +3588,10 @@
         <v>44108</v>
       </c>
       <c r="B83" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="C83" t="s">
-        <v>135</v>
+        <v>112</v>
       </c>
       <c r="D83">
         <v>27.452604600000001</v>
@@ -3588,10 +3600,10 @@
         <v>90.067492799999997</v>
       </c>
       <c r="F83" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J83" t="s">
-        <v>135</v>
+        <v>112</v>
       </c>
       <c r="K83">
         <v>4</v>
@@ -3602,10 +3614,10 @@
         <v>44360</v>
       </c>
       <c r="B84" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C84" t="s">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="D84">
         <v>27.610600000000002</v>
@@ -3617,7 +3629,7 @@
         <v>13</v>
       </c>
       <c r="G84" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K84">
         <v>1</v>
@@ -3628,10 +3640,10 @@
         <v>44362</v>
       </c>
       <c r="B85" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C85" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="D85">
         <v>27.499400000000001</v>
@@ -3643,10 +3655,10 @@
         <v>13</v>
       </c>
       <c r="G85" t="s">
-        <v>138</v>
+        <v>160</v>
       </c>
       <c r="H85" t="s">
-        <v>139</v>
+        <v>115</v>
       </c>
       <c r="K85">
         <v>3</v>
@@ -3657,10 +3669,10 @@
         <v>44362</v>
       </c>
       <c r="B86" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C86" t="s">
-        <v>140</v>
+        <v>116</v>
       </c>
       <c r="D86">
         <v>27.530100000000001</v>
@@ -3672,7 +3684,7 @@
         <v>13</v>
       </c>
       <c r="J86" t="s">
-        <v>140</v>
+        <v>116</v>
       </c>
       <c r="K86">
         <v>4</v>
@@ -3683,10 +3695,10 @@
         <v>44362</v>
       </c>
       <c r="B87" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C87" t="s">
-        <v>141</v>
+        <v>117</v>
       </c>
       <c r="D87">
         <v>27.557600000000001</v>
@@ -3698,7 +3710,7 @@
         <v>13</v>
       </c>
       <c r="G87" t="s">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="K87">
         <v>1</v>
@@ -3709,10 +3721,10 @@
         <v>44363</v>
       </c>
       <c r="B88" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C88" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="D88">
         <v>28.051500000000001</v>
@@ -3721,10 +3733,13 @@
         <v>89.634299999999996</v>
       </c>
       <c r="F88" t="s">
-        <v>143</v>
+        <v>13</v>
+      </c>
+      <c r="G88" t="s">
+        <v>162</v>
       </c>
       <c r="J88" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="K88">
         <v>4</v>
@@ -3735,10 +3750,10 @@
         <v>44416</v>
       </c>
       <c r="B89" t="s">
-        <v>144</v>
+        <v>118</v>
       </c>
       <c r="C89" t="s">
-        <v>145</v>
+        <v>119</v>
       </c>
       <c r="D89">
         <v>27.613900000000001</v>
@@ -3747,10 +3762,10 @@
         <v>91.508600000000001</v>
       </c>
       <c r="F89" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J89" t="s">
-        <v>145</v>
+        <v>119</v>
       </c>
       <c r="K89">
         <v>4</v>
@@ -3761,10 +3776,10 @@
         <v>44420</v>
       </c>
       <c r="B90" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="C90" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="D90">
         <v>26.870556000000001</v>
@@ -3776,7 +3791,7 @@
         <v>13</v>
       </c>
       <c r="G90" t="s">
-        <v>146</v>
+        <v>120</v>
       </c>
       <c r="K90">
         <v>3</v>
@@ -3787,10 +3802,10 @@
         <v>44433</v>
       </c>
       <c r="B91" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C91" t="s">
-        <v>147</v>
+        <v>121</v>
       </c>
       <c r="D91">
         <v>26.8627</v>
@@ -3799,10 +3814,10 @@
         <v>90.271699999999996</v>
       </c>
       <c r="F91" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J91" t="s">
-        <v>147</v>
+        <v>121</v>
       </c>
       <c r="K91">
         <v>4</v>
@@ -3813,10 +3828,10 @@
         <v>44433</v>
       </c>
       <c r="B92" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="C92" t="s">
-        <v>148</v>
+        <v>122</v>
       </c>
       <c r="D92">
         <v>26.870556000000001</v>
@@ -3828,7 +3843,7 @@
         <v>13</v>
       </c>
       <c r="G92" t="s">
-        <v>149</v>
+        <v>123</v>
       </c>
       <c r="K92">
         <v>3</v>
@@ -3839,10 +3854,10 @@
         <v>44433</v>
       </c>
       <c r="B93" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C93" t="s">
-        <v>148</v>
+        <v>122</v>
       </c>
       <c r="D93">
         <v>27.991900000000001</v>
@@ -3854,7 +3869,7 @@
         <v>13</v>
       </c>
       <c r="G93" t="s">
-        <v>149</v>
+        <v>123</v>
       </c>
       <c r="K93">
         <v>3</v>
@@ -3865,10 +3880,10 @@
         <v>44434</v>
       </c>
       <c r="B94" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C94" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="D94">
         <v>28.051500000000001</v>
@@ -3877,10 +3892,10 @@
         <v>89.634299999999996</v>
       </c>
       <c r="F94" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J94" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="K94">
         <v>4</v>
@@ -3891,10 +3906,10 @@
         <v>44488</v>
       </c>
       <c r="B95" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C95" t="s">
-        <v>150</v>
+        <v>124</v>
       </c>
       <c r="D95">
         <v>27.029183199999999</v>
@@ -3906,7 +3921,7 @@
         <v>13</v>
       </c>
       <c r="G95" t="s">
-        <v>151</v>
+        <v>125</v>
       </c>
       <c r="K95">
         <v>3</v>
@@ -3917,10 +3932,10 @@
         <v>44749</v>
       </c>
       <c r="B96" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C96" t="s">
-        <v>152</v>
+        <v>126</v>
       </c>
       <c r="D96">
         <v>27.502600000000001</v>
@@ -3932,7 +3947,7 @@
         <v>13</v>
       </c>
       <c r="G96" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K96">
         <v>1</v>
@@ -3943,10 +3958,10 @@
         <v>44749</v>
       </c>
       <c r="B97" t="s">
-        <v>112</v>
+        <v>92</v>
       </c>
       <c r="C97" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="D97">
         <v>27.0246</v>
@@ -3955,10 +3970,10 @@
         <v>90.124600000000001</v>
       </c>
       <c r="F97" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G97" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="K97">
         <v>1</v>
@@ -3969,10 +3984,10 @@
         <v>44749</v>
       </c>
       <c r="B98" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C98" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="D98">
         <v>27.6678</v>
@@ -3984,7 +3999,7 @@
         <v>13</v>
       </c>
       <c r="G98" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K98">
         <v>1</v>
@@ -3995,10 +4010,10 @@
         <v>44749</v>
       </c>
       <c r="B99" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C99" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D99">
         <v>26.8627</v>
@@ -4007,10 +4022,10 @@
         <v>90.271699999999996</v>
       </c>
       <c r="F99" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G99" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="K99">
         <v>1</v>
@@ -4021,10 +4036,10 @@
         <v>44749</v>
       </c>
       <c r="B100" t="s">
-        <v>154</v>
+        <v>127</v>
       </c>
       <c r="C100" t="s">
-        <v>155</v>
+        <v>128</v>
       </c>
       <c r="D100">
         <v>27.045000000000002</v>
@@ -4036,7 +4051,7 @@
         <v>13</v>
       </c>
       <c r="G100" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K100">
         <v>1</v>
@@ -4047,10 +4062,10 @@
         <v>44749</v>
       </c>
       <c r="B101" t="s">
-        <v>144</v>
+        <v>118</v>
       </c>
       <c r="C101" t="s">
-        <v>156</v>
+        <v>129</v>
       </c>
       <c r="D101">
         <v>27.613900000000001</v>
@@ -4062,7 +4077,7 @@
         <v>13</v>
       </c>
       <c r="G101" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K101">
         <v>1</v>
@@ -4073,10 +4088,10 @@
         <v>44749</v>
       </c>
       <c r="B102" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C102" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="D102">
         <v>27.333200000000001</v>
@@ -4088,7 +4103,7 @@
         <v>13</v>
       </c>
       <c r="G102" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K102">
         <v>1</v>
@@ -4099,10 +4114,10 @@
         <v>44749</v>
       </c>
       <c r="B103" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="C103" t="s">
-        <v>119</v>
+        <v>98</v>
       </c>
       <c r="D103">
         <v>27.267600000000002</v>
@@ -4114,7 +4129,7 @@
         <v>13</v>
       </c>
       <c r="G103" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K103">
         <v>1</v>
@@ -4128,7 +4143,7 @@
         <v>11</v>
       </c>
       <c r="C104" t="s">
-        <v>157</v>
+        <v>130</v>
       </c>
       <c r="D104">
         <v>27.549399999999999</v>
@@ -4140,7 +4155,7 @@
         <v>13</v>
       </c>
       <c r="G104" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K104">
         <v>1</v>
@@ -4151,10 +4166,10 @@
         <v>44749</v>
       </c>
       <c r="B105" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="C105" t="s">
-        <v>158</v>
+        <v>131</v>
       </c>
       <c r="D105">
         <v>27.27</v>
@@ -4166,7 +4181,7 @@
         <v>13</v>
       </c>
       <c r="G105" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K105">
         <v>1</v>
@@ -4177,10 +4192,10 @@
         <v>44749</v>
       </c>
       <c r="B106" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C106" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D106">
         <v>26.805499999999999</v>
@@ -4189,10 +4204,10 @@
         <v>91.503600000000006</v>
       </c>
       <c r="F106" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G106" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="K106">
         <v>1</v>
@@ -4203,10 +4218,10 @@
         <v>44834</v>
       </c>
       <c r="B107" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C107" t="s">
-        <v>159</v>
+        <v>132</v>
       </c>
       <c r="D107">
         <v>27.667870000000001</v>
@@ -4218,7 +4233,7 @@
         <v>13</v>
       </c>
       <c r="G107" t="s">
-        <v>160</v>
+        <v>133</v>
       </c>
       <c r="K107">
         <v>3</v>
@@ -4229,7 +4244,7 @@
         <v>45120</v>
       </c>
       <c r="C108" t="s">
-        <v>161</v>
+        <v>134</v>
       </c>
       <c r="D108">
         <v>26.861529999999998</v>
@@ -4241,7 +4256,7 @@
         <v>13</v>
       </c>
       <c r="G108" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="K108">
         <v>3</v>
@@ -4252,10 +4267,10 @@
         <v>45127</v>
       </c>
       <c r="B109" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C109" t="s">
-        <v>163</v>
+        <v>135</v>
       </c>
       <c r="D109">
         <v>27.667870000000001</v>
@@ -4267,7 +4282,7 @@
         <v>13</v>
       </c>
       <c r="G109" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K109">
         <v>3</v>
@@ -4278,10 +4293,10 @@
         <v>45163</v>
       </c>
       <c r="B110" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="C110" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="D110">
         <v>27.452604600000001</v>
@@ -4290,7 +4305,7 @@
         <v>90.067492799999997</v>
       </c>
       <c r="F110" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G110" t="s">
         <v>166</v>
@@ -4304,10 +4319,10 @@
         <v>45514</v>
       </c>
       <c r="B111" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C111" t="s">
-        <v>167</v>
+        <v>137</v>
       </c>
       <c r="D111">
         <v>27.466090000000001</v>
@@ -4316,10 +4331,10 @@
         <v>89.641909999999996</v>
       </c>
       <c r="F111" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G111" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K111">
         <v>3</v>
@@ -4330,10 +4345,10 @@
         <v>45810</v>
       </c>
       <c r="B112" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C112" t="s">
-        <v>169</v>
+        <v>138</v>
       </c>
       <c r="D112">
         <v>27.591370000000001</v>
@@ -4345,7 +4360,7 @@
         <v>13</v>
       </c>
       <c r="G112" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="K112">
         <v>3</v>
@@ -4356,10 +4371,10 @@
         <v>45810</v>
       </c>
       <c r="B113" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C113" t="s">
-        <v>169</v>
+        <v>138</v>
       </c>
       <c r="D113">
         <v>28.018588600000001</v>
@@ -4371,7 +4386,7 @@
         <v>13</v>
       </c>
       <c r="G113" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="K113">
         <v>3</v>
@@ -4382,10 +4397,10 @@
         <v>45830</v>
       </c>
       <c r="B114" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C114" t="s">
-        <v>171</v>
+        <v>139</v>
       </c>
       <c r="D114">
         <v>27.591370000000001</v>
@@ -4397,7 +4412,7 @@
         <v>13</v>
       </c>
       <c r="G114" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="K114">
         <v>3</v>
@@ -4405,5 +4420,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>